<commit_message>
feat(skydive): 자세를 잡으려면 필요한 발밑 여유(pose_clearance)
젤다는 공중에 충분히 떠 있을 때만 자세를 잡을 수 있다 — 서서 패러세일을
펴거나 지면 코앞에서 다이브에 들어갈 수는 없다. 20m로 시작한다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnnTW5GzPD2EEBt127mrs7
</commit_message>
<xml_diff>
--- a/table/Datas/#SkydiveConfig.xlsx
+++ b/table/Datas/#SkydiveConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -532,6 +532,11 @@
           <t>jump_power</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>pose_clearance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -649,6 +654,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -771,6 +781,11 @@
       <c r="W4" t="inlineStr">
         <is>
           <t>jump_power</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>pose_clearance</t>
         </is>
       </c>
     </row>
@@ -840,6 +855,9 @@
       </c>
       <c r="W5" t="n">
         <v>11</v>
+      </c>
+      <c r="X5" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(skydive): 하강 감속(fall_brake)을 가속과 따로 둔다
패러세일을 펴도 하강이 중력과 같은 비율(29)로만 줄어 60에서 6까지 1.9초가
걸렸다. 낙하산이 아니라 그냥 천천히 느려지는 것이다. 공기 저항은 면적이
커지면 급격히 커지므로 커지는 쪽과 줄어드는 쪽이 원래 대칭이 아니다.

150으로 시작한다 — 60에서 6까지 0.36초.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnnTW5GzPD2EEBt127mrs7
</commit_message>
<xml_diff>
--- a/table/Datas/#SkydiveConfig.xlsx
+++ b/table/Datas/#SkydiveConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,6 +537,11 @@
           <t>pose_clearance</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>fall_brake</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -659,6 +664,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -786,6 +796,11 @@
       <c r="X4" t="inlineStr">
         <is>
           <t>pose_clearance</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>fall_brake</t>
         </is>
       </c>
     </row>
@@ -858,6 +873,9 @@
       </c>
       <c r="X5" t="n">
         <v>5</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(skydive): TbSkydiveConfig에 restitution 열을 더한다
캐릭터 몸끼리 부딪혔을 때의 반발계수(0.35)를 마스터데이터에서 읽도록 한다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#SkydiveConfig.xlsx
+++ b/table/Datas/#SkydiveConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AD5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,6 +562,11 @@
           <t>landing_lethal_speed</t>
         </is>
       </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>restitution</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -709,6 +714,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -861,6 +871,11 @@
       <c r="AC4" t="inlineStr">
         <is>
           <t>landing_lethal_speed</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>restitution</t>
         </is>
       </c>
     </row>
@@ -948,6 +963,9 @@
       </c>
       <c r="AC5" t="n">
         <v>15</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>